<commit_message>
📊 Auto scan: 2026-09-27
</commit_message>
<xml_diff>
--- a/archive/2026-09-28/report.xlsx
+++ b/archive/2026-09-28/report.xlsx
@@ -603,7 +603,7 @@
   <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="55" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
@@ -652,7 +652,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>엔비디아</t>
+          <t>콜럼버스 크루 대 인터 마이애미</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -681,7 +681,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>alvin kamara</t>
+          <t>dak prescott</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -710,7 +710,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>michelle randolph</t>
+          <t>ravens head coach</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -739,7 +739,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>weather</t>
+          <t>나는 solo</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -768,7 +768,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>차범근</t>
+          <t>식중독</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -797,7 +797,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>mike washington jr.</t>
+          <t>dak prescott wife</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -826,7 +826,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>chris moore</t>
+          <t>nfc north</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -855,7 +855,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>김량하</t>
+          <t>klasemen tim nasional sepak bola norwegia vs portugal</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -884,7 +884,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>inter miami vs columbus</t>
+          <t>chase young</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -913,7 +913,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>퇴직</t>
+          <t>권상우</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -942,7 +942,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>청원</t>
+          <t>엔비디아</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -971,7 +971,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>baker mayfield</t>
+          <t>cook political report</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1025,7 +1025,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>이슬람 혁명 수비대</t>
+          <t>weather</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1054,7 +1054,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>mystics vs dream</t>
+          <t>cody white</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1083,7 +1083,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>엘링 홀란</t>
+          <t>차범근</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1112,7 +1112,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>haiti vs costa rica</t>
+          <t>trey mcbride</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1141,7 +1141,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>사과</t>
+          <t>김량하</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1195,7 +1195,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>who won the presidents cup</t>
+          <t>ncis</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1224,7 +1224,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>nations league</t>
+          <t>퇴직</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1253,7 +1253,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>shaq</t>
+          <t>broncos game today</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -8953,7 +8953,7 @@
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
     <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="27" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
     <col width="60" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
@@ -9049,7 +9049,7 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>62.1</v>
+        <v>60</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -9060,7 +9060,7 @@
         <v>60</v>
       </c>
       <c r="I2" t="n">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="J2" t="n">
         <v>25</v>
@@ -9070,12 +9070,12 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>엔비디아, haiti vs costa rica</t>
+          <t>엔비디아</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>[테마: AI/반도체] 거래량 시그널 60점 (2주avg/4-8주avg = 2.04, 2주/2-4주 = 1.09). 트렌드 시그널 86점 — 매칭 키워드: 엔비디아(google, 100점), haiti vs costa rica(google, 72점). 동일 테마 동시통과 1종목(밀집도 25점). 종목 근거: 특화 파운드리</t>
+          <t>[테마: AI/반도체] 거래량 시그널 60점 (2주avg/4-8주avg = 2.04, 2주/2-4주 = 1.09). 트렌드 시그널 80점 — 매칭 키워드: 엔비디아(google, 80점). 동일 테마 동시통과 1종목(밀집도 25점). 종목 근거: 특화 파운드리</t>
         </is>
       </c>
     </row>

</xml_diff>